<commit_message>
Actualización del catálogo y ajustes de diseño 14 Abril V2
</commit_message>
<xml_diff>
--- a/casa_14042028.xlsx
+++ b/casa_14042028.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hans_\OneDrive\Escritorio\Projectos\Desarrollos FEr\gestioninmobiliargalindo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{81EB9F2B-E603-4D7A-BB48-5EB81C280C0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{136A3F00-ADEB-4C4D-888F-49F3B083A181}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1882,8 +1882,12 @@
       <c r="H17" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="I17" s="9"/>
-      <c r="J17" s="9"/>
+      <c r="I17" s="9">
+        <v>150</v>
+      </c>
+      <c r="J17" s="9">
+        <v>100</v>
+      </c>
       <c r="K17" s="9">
         <v>3</v>
       </c>

</xml_diff>